<commit_message>
UPDATE: 7 class complete
</commit_message>
<xml_diff>
--- a/docs/任务计划-吴正日.xlsx
+++ b/docs/任务计划-吴正日.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaron/Documents/Projects/mingtai/traffic-light/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0FCD3B-A4E2-2E4A-8FF7-1DE0084ADF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDA5A5B-635A-2D4B-A117-A840165F369A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="860" windowWidth="29840" windowHeight="18560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="61">
   <si>
     <t>底软</t>
   </si>
@@ -144,9 +144,6 @@
     <t>5/11–5/15</t>
   </si>
   <si>
-    <t>数据流水线升级（9类）</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -202,13 +199,19 @@
   </si>
   <si>
     <t>B = 基于自采商用数据训练</t>
+  </si>
+  <si>
+    <t>已完成</t>
+  </si>
+  <si>
+    <t>数据流水线升级（7类）</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -273,6 +276,13 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -440,7 +450,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -511,6 +521,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1144,10 +1157,10 @@
     </row>
     <row r="5" spans="1:35">
       <c r="A5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>40</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>41</v>
       </c>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -1179,13 +1192,16 @@
       <c r="AD5" s="16"/>
       <c r="AE5" s="16"/>
       <c r="AF5" s="16"/>
+      <c r="AG5" s="33" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="6" spans="1:35">
       <c r="A6" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="18"/>
       <c r="D6" s="18"/>
@@ -1217,13 +1233,16 @@
       <c r="AD6" s="16"/>
       <c r="AE6" s="16"/>
       <c r="AF6" s="16"/>
+      <c r="AG6" s="33" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="7" spans="1:35">
       <c r="A7" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>43</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>44</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="19"/>
@@ -1258,10 +1277,10 @@
     </row>
     <row r="8" spans="1:35">
       <c r="A8" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
@@ -1296,10 +1315,10 @@
     </row>
     <row r="9" spans="1:35">
       <c r="A9" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -1334,10 +1353,10 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>47</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>48</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
@@ -1372,10 +1391,10 @@
     </row>
     <row r="11" spans="1:35">
       <c r="A11" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
@@ -1410,10 +1429,10 @@
     </row>
     <row r="12" spans="1:35">
       <c r="A12" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -1448,10 +1467,10 @@
     </row>
     <row r="13" spans="1:35">
       <c r="A13" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -1486,10 +1505,10 @@
     </row>
     <row r="14" spans="1:35">
       <c r="A14" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
@@ -1524,38 +1543,38 @@
     </row>
     <row r="16" spans="1:35" ht="16">
       <c r="A16" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="I16" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="I16" s="24" t="s">
-        <v>54</v>
-      </c>
       <c r="AF16" s="24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>